<commit_message>
Add scenario test sets TS6-TS12 and a module-wise test-case list
TS6-TS10 and TS12 are chained lead + signal files that run Prospecting ->
Scoring -> Micro-segments -> For Review, each designed around one area:
segment boundaries, scoring and fit boundaries, contactability and channel,
For Review routing, and rep ownership; TS12 is a realistic 60-account list.
TS11 re-scores TS1 on five dates. run_scenarios.js checks every account
against the result it was designed for; three known gaps are marked.
POC_Test_Cases.xlsx lists 163 cases by module with expected results.
TS4 is now marked optional.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XiLXGU1oR1hNbNccyNpRo1
</commit_message>
<xml_diff>
--- a/test-data/poc-test-sets/TS4_Microsegments_from_file.xlsx
+++ b/test-data/poc-test-sets/TS4_Microsegments_from_file.xlsx
@@ -2189,7 +2189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -2210,31 +2210,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Optional: micro-segments normally come from Scoring (TS1, TS6 to TS10 test that). Run this set only if lists scored outside the POC are in scope.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>In Micro-segments &amp; NBA choose to upload a file, set the scoring date to 2026-10-20, and upload this file.</t>
-        </is>
-      </c>
+      <c r="A4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Expect 12 rows read, 2 rejected, 10 accounts, and 2 segments: Inquiry 4 and Modernisation 3.</t>
+          <t>In Micro-segments &amp; NBA choose to upload a file, set the scoring date to 2026-10-20, and upload this file.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Johor Aromatics, Rayong Olefins and Cilacap Refining get no segment, because fewer than 3 accounts share their strongest signal. They go to For Review.</t>
+          <t>Expect 12 rows read, 2 rejected, 10 accounts, and 2 segments: Inquiry 4 and Modernisation 3.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Johor Aromatics, Rayong Olefins and Cilacap Refining get no segment, because fewer than 3 accounts share their strongest signal. They go to For Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Compare each row with "Answer key".</t>
         </is>

</xml_diff>